<commit_message>
Update filtered yeast peptide matrix and group QC figures
</commit_message>
<xml_diff>
--- a/sample-QC-InternalQC-HELP_yeast.xlsx
+++ b/sample-QC-InternalQC-HELP_yeast.xlsx
@@ -715,11 +715,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DF3"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:BX3"/>
+  <sheetFormatPr defaultRowHeight="14" ns3:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:110" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:76" s="1" customFormat="1" ns3:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -739,316 +739,214 @@
         <v>1</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>42</v>
+        <v>65</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="AX1" s="1" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="AZ1" s="1" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="BA1" s="1" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="BB1" s="1" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="BC1" s="1" t="s">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="BD1" s="1" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="BE1" s="1" t="s">
-        <v>51</v>
+        <v>81</v>
       </c>
       <c r="BF1" s="1" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="BG1" s="1" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="BH1" s="1" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="BI1" s="1" t="s">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="BJ1" s="1" t="s">
-        <v>56</v>
+        <v>89</v>
       </c>
       <c r="BK1" s="1" t="s">
-        <v>57</v>
+        <v>90</v>
       </c>
       <c r="BL1" s="1" t="s">
-        <v>58</v>
+        <v>91</v>
       </c>
       <c r="BM1" s="1" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="BN1" s="1" t="s">
-        <v>60</v>
+        <v>94</v>
       </c>
       <c r="BO1" s="1" t="s">
-        <v>61</v>
+        <v>95</v>
       </c>
       <c r="BP1" s="1" t="s">
-        <v>62</v>
+        <v>96</v>
       </c>
       <c r="BQ1" s="1" t="s">
-        <v>63</v>
+        <v>97</v>
       </c>
       <c r="BR1" s="1" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="BS1" s="1" t="s">
-        <v>65</v>
+        <v>99</v>
       </c>
       <c r="BT1" s="1" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="BU1" s="1" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="BV1" s="1" t="s">
-        <v>68</v>
+        <v>102</v>
       </c>
       <c r="BW1" s="1" t="s">
-        <v>69</v>
+        <v>103</v>
       </c>
       <c r="BX1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="BY1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="BZ1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="CA1" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="CB1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="CC1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="CD1" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="CE1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="CF1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="CG1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="CH1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="CI1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="CJ1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="CK1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="CL1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="CM1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="CN1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="CO1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="CP1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="CQ1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="CR1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="CS1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="CT1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="CU1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="CV1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="CW1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="CX1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="CY1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="CZ1" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="DA1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="DB1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="DC1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="DD1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="DE1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="DF1" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:110" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:76" ns3:dyDescent="0.25">
       <c r="A2" t="s">
         <v>105</v>
       </c>
@@ -1071,316 +969,214 @@
         <v>20500</v>
       </c>
       <c r="H2">
-        <v>11158671</v>
+        <v>13146627</v>
       </c>
       <c r="I2">
-        <v>70584851</v>
+        <v>22912528</v>
       </c>
       <c r="J2">
-        <v>13146627</v>
+        <v>8014632</v>
       </c>
       <c r="K2">
-        <v>31793140</v>
+        <v>7857983</v>
       </c>
       <c r="L2">
-        <v>22912528</v>
+        <v>12443384</v>
       </c>
       <c r="M2">
-        <v>12834903</v>
+        <v>15121761</v>
       </c>
       <c r="N2">
-        <v>8014632</v>
+        <v>16725424</v>
       </c>
       <c r="O2">
-        <v>53038169</v>
+        <v>25120234</v>
       </c>
       <c r="P2">
-        <v>7857983</v>
+        <v>11431256</v>
       </c>
       <c r="Q2">
-        <v>12443384</v>
+        <v>22022385</v>
       </c>
       <c r="R2">
-        <v>61812752</v>
+        <v>14567788</v>
       </c>
       <c r="S2">
-        <v>15121761</v>
+        <v>11558852</v>
       </c>
       <c r="T2">
-        <v>53147867</v>
+        <v>15712141</v>
       </c>
       <c r="U2">
-        <v>16725424</v>
+        <v>13868633</v>
       </c>
       <c r="V2">
-        <v>44244108</v>
+        <v>11453913</v>
       </c>
       <c r="W2">
-        <v>25120234</v>
+        <v>14659677</v>
       </c>
       <c r="X2">
-        <v>66360282</v>
+        <v>13432771</v>
       </c>
       <c r="Y2">
-        <v>11431256</v>
+        <v>20139547</v>
       </c>
       <c r="Z2">
-        <v>22022385</v>
+        <v>14833377</v>
       </c>
       <c r="AA2">
-        <v>14567788</v>
+        <v>9354858</v>
       </c>
       <c r="AB2">
-        <v>11558852</v>
+        <v>7828859</v>
       </c>
       <c r="AC2">
-        <v>60630051</v>
+        <v>34339437</v>
       </c>
       <c r="AD2">
-        <v>15712141</v>
+        <v>13897133</v>
       </c>
       <c r="AE2">
-        <v>31050461</v>
+        <v>12696559</v>
       </c>
       <c r="AF2">
-        <v>55531970</v>
+        <v>21843511</v>
       </c>
       <c r="AG2">
-        <v>57534514</v>
+        <v>13536776</v>
       </c>
       <c r="AH2">
-        <v>13868633</v>
+        <v>18589199</v>
       </c>
       <c r="AI2">
-        <v>11453913</v>
+        <v>20252458</v>
       </c>
       <c r="AJ2">
-        <v>14659677</v>
+        <v>14389928</v>
       </c>
       <c r="AK2">
-        <v>13432771</v>
+        <v>8235159</v>
       </c>
       <c r="AL2">
-        <v>20139547</v>
+        <v>14043741</v>
       </c>
       <c r="AM2">
-        <v>14833377</v>
+        <v>12140629</v>
       </c>
       <c r="AN2">
-        <v>9354858</v>
+        <v>15302671</v>
       </c>
       <c r="AO2">
-        <v>7828859</v>
+        <v>15491034</v>
       </c>
       <c r="AP2">
-        <v>34339437</v>
+        <v>11642105</v>
       </c>
       <c r="AQ2">
-        <v>13897133</v>
+        <v>13820024</v>
       </c>
       <c r="AR2">
-        <v>12696559</v>
+        <v>10471617</v>
       </c>
       <c r="AS2">
-        <v>29214835</v>
+        <v>11719270</v>
       </c>
       <c r="AT2">
-        <v>10002903</v>
+        <v>21330010</v>
       </c>
       <c r="AU2">
-        <v>12930782</v>
+        <v>12660732</v>
       </c>
       <c r="AV2">
-        <v>31728275</v>
+        <v>22129235</v>
       </c>
       <c r="AW2">
-        <v>21843511</v>
+        <v>14904911</v>
       </c>
       <c r="AX2">
-        <v>13536776</v>
+        <v>9775965</v>
       </c>
       <c r="AY2">
-        <v>58923343</v>
+        <v>9832312</v>
       </c>
       <c r="AZ2">
-        <v>18589199</v>
+        <v>18401646</v>
       </c>
       <c r="BA2">
-        <v>20252458</v>
+        <v>8977735</v>
       </c>
       <c r="BB2">
-        <v>14389928</v>
+        <v>12829574</v>
       </c>
       <c r="BC2">
-        <v>8235159</v>
+        <v>10800499</v>
       </c>
       <c r="BD2">
-        <v>67044369</v>
+        <v>11921788</v>
       </c>
       <c r="BE2">
-        <v>60925840</v>
+        <v>16467581</v>
       </c>
       <c r="BF2">
-        <v>14043741</v>
+        <v>15870740</v>
       </c>
       <c r="BG2">
-        <v>12140629</v>
+        <v>18164983</v>
       </c>
       <c r="BH2">
-        <v>69309459</v>
+        <v>7837749</v>
       </c>
       <c r="BI2">
-        <v>15302671</v>
+        <v>16897755</v>
       </c>
       <c r="BJ2">
-        <v>15491034</v>
+        <v>15277353</v>
       </c>
       <c r="BK2">
-        <v>54453128</v>
+        <v>26392961</v>
       </c>
       <c r="BL2">
-        <v>11642105</v>
+        <v>19808787</v>
       </c>
       <c r="BM2">
-        <v>13820024</v>
+        <v>16172659</v>
       </c>
       <c r="BN2">
-        <v>10471617</v>
+        <v>12880022</v>
       </c>
       <c r="BO2">
-        <v>53169939</v>
+        <v>20460708</v>
       </c>
       <c r="BP2">
-        <v>11719270</v>
+        <v>11520465</v>
       </c>
       <c r="BQ2">
-        <v>21330010</v>
+        <v>10716086</v>
       </c>
       <c r="BR2">
-        <v>12660732</v>
+        <v>13001424</v>
       </c>
       <c r="BS2">
-        <v>22129235</v>
+        <v>11619387</v>
       </c>
       <c r="BT2">
-        <v>53663887</v>
+        <v>21343619</v>
       </c>
       <c r="BU2">
-        <v>44721486</v>
+        <v>16268736</v>
       </c>
       <c r="BV2">
-        <v>14904911</v>
+        <v>18051601</v>
       </c>
       <c r="BW2">
-        <v>58089333</v>
+        <v>14585498</v>
       </c>
       <c r="BX2">
-        <v>9775965</v>
-      </c>
-      <c r="BY2">
-        <v>9832312</v>
-      </c>
-      <c r="BZ2">
-        <v>18401646</v>
-      </c>
-      <c r="CA2">
-        <v>54749969</v>
-      </c>
-      <c r="CB2">
-        <v>31509385</v>
-      </c>
-      <c r="CC2">
-        <v>54146467</v>
-      </c>
-      <c r="CD2">
-        <v>47598180</v>
-      </c>
-      <c r="CE2">
-        <v>8977735</v>
-      </c>
-      <c r="CF2">
-        <v>12829574</v>
-      </c>
-      <c r="CG2">
-        <v>10800499</v>
-      </c>
-      <c r="CH2">
-        <v>11921788</v>
-      </c>
-      <c r="CI2">
-        <v>16467581</v>
-      </c>
-      <c r="CJ2">
-        <v>57358430</v>
-      </c>
-      <c r="CK2">
-        <v>15870740</v>
-      </c>
-      <c r="CL2">
-        <v>10761747</v>
-      </c>
-      <c r="CM2">
-        <v>31595965</v>
-      </c>
-      <c r="CN2">
-        <v>18164983</v>
-      </c>
-      <c r="CO2">
-        <v>7837749</v>
-      </c>
-      <c r="CP2">
-        <v>16897755</v>
-      </c>
-      <c r="CQ2">
-        <v>15277353</v>
-      </c>
-      <c r="CR2">
-        <v>26392961</v>
-      </c>
-      <c r="CS2">
-        <v>19808787</v>
-      </c>
-      <c r="CT2">
-        <v>16172659</v>
-      </c>
-      <c r="CU2">
-        <v>33767927</v>
-      </c>
-      <c r="CV2">
-        <v>12880022</v>
-      </c>
-      <c r="CW2">
-        <v>20460708</v>
-      </c>
-      <c r="CX2">
-        <v>11520465</v>
-      </c>
-      <c r="CY2">
-        <v>10716086</v>
-      </c>
-      <c r="CZ2">
-        <v>13001424</v>
-      </c>
-      <c r="DA2">
-        <v>11619387</v>
-      </c>
-      <c r="DB2">
-        <v>21343619</v>
-      </c>
-      <c r="DC2">
-        <v>16268736</v>
-      </c>
-      <c r="DD2">
-        <v>18051601</v>
-      </c>
-      <c r="DE2">
-        <v>14585498</v>
-      </c>
-      <c r="DF2">
         <v>15285354</v>
       </c>
     </row>
-    <row r="3" spans="1:110" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:76" ns3:dyDescent="0.25">
       <c r="A3" t="s">
         <v>106</v>
       </c>
@@ -1403,312 +1199,210 @@
         <v>22375</v>
       </c>
       <c r="H3">
-        <v>8872055</v>
+        <v>10246427</v>
       </c>
       <c r="I3">
-        <v>62455425</v>
+        <v>19351265</v>
       </c>
       <c r="J3">
-        <v>10246427</v>
+        <v>6286801</v>
       </c>
       <c r="K3">
-        <v>22789394</v>
+        <v>6227158</v>
       </c>
       <c r="L3">
-        <v>19351265</v>
+        <v>9749163</v>
       </c>
       <c r="M3">
-        <v>9781057</v>
+        <v>11562175</v>
       </c>
       <c r="N3">
-        <v>6286801</v>
+        <v>12932828</v>
       </c>
       <c r="O3">
-        <v>50023316</v>
+        <v>21158085</v>
       </c>
       <c r="P3">
-        <v>6227158</v>
+        <v>8520438</v>
       </c>
       <c r="Q3">
-        <v>9749163</v>
+        <v>18180217</v>
       </c>
       <c r="R3">
-        <v>51393975</v>
+        <v>11570083</v>
       </c>
       <c r="S3">
-        <v>11562175</v>
+        <v>8725928</v>
       </c>
       <c r="T3">
-        <v>46489162</v>
+        <v>12866849</v>
       </c>
       <c r="U3">
-        <v>12932828</v>
+        <v>10771856</v>
       </c>
       <c r="V3">
-        <v>40505531</v>
+        <v>8584355</v>
       </c>
       <c r="W3">
-        <v>21158085</v>
+        <v>11917285</v>
       </c>
       <c r="X3">
-        <v>50197142</v>
+        <v>10565249</v>
       </c>
       <c r="Y3">
-        <v>8520438</v>
+        <v>17405820</v>
       </c>
       <c r="Z3">
-        <v>18180217</v>
+        <v>11237650</v>
       </c>
       <c r="AA3">
-        <v>11570083</v>
+        <v>7388464</v>
       </c>
       <c r="AB3">
-        <v>8725928</v>
+        <v>5662526</v>
       </c>
       <c r="AC3">
-        <v>51992570</v>
+        <v>27938691</v>
       </c>
       <c r="AD3">
-        <v>12866849</v>
+        <v>11195894</v>
       </c>
       <c r="AE3">
-        <v>21917035</v>
+        <v>9526324</v>
       </c>
       <c r="AF3">
-        <v>49146936</v>
+        <v>16883101</v>
       </c>
       <c r="AG3">
-        <v>48426912</v>
+        <v>10055299</v>
       </c>
       <c r="AH3">
-        <v>10771856</v>
+        <v>15030792</v>
       </c>
       <c r="AI3">
-        <v>8584355</v>
+        <v>17333300</v>
       </c>
       <c r="AJ3">
-        <v>11917285</v>
+        <v>10897736</v>
       </c>
       <c r="AK3">
-        <v>10565249</v>
+        <v>5566103</v>
       </c>
       <c r="AL3">
-        <v>17405820</v>
+        <v>10541701</v>
       </c>
       <c r="AM3">
-        <v>11237650</v>
+        <v>9106435</v>
       </c>
       <c r="AN3">
-        <v>7388464</v>
+        <v>12045156</v>
       </c>
       <c r="AO3">
-        <v>5662526</v>
+        <v>12929595</v>
       </c>
       <c r="AP3">
-        <v>27938691</v>
+        <v>8756328</v>
       </c>
       <c r="AQ3">
-        <v>11195894</v>
+        <v>10992686</v>
       </c>
       <c r="AR3">
-        <v>9526324</v>
+        <v>8025234</v>
       </c>
       <c r="AS3">
-        <v>22146080</v>
+        <v>8796815</v>
       </c>
       <c r="AT3">
-        <v>7515120</v>
+        <v>17170707</v>
       </c>
       <c r="AU3">
-        <v>9270957</v>
+        <v>10258250</v>
       </c>
       <c r="AV3">
-        <v>22382046</v>
+        <v>18579886</v>
       </c>
       <c r="AW3">
-        <v>16883101</v>
+        <v>11993548</v>
       </c>
       <c r="AX3">
-        <v>10055299</v>
+        <v>7522157</v>
       </c>
       <c r="AY3">
-        <v>49749620</v>
+        <v>7523813</v>
       </c>
       <c r="AZ3">
-        <v>15030792</v>
+        <v>14002461</v>
       </c>
       <c r="BA3">
-        <v>17333300</v>
+        <v>6514265</v>
       </c>
       <c r="BB3">
-        <v>10897736</v>
+        <v>9523452</v>
       </c>
       <c r="BC3">
-        <v>5566103</v>
+        <v>7892769</v>
       </c>
       <c r="BD3">
-        <v>54870939</v>
+        <v>8517468</v>
       </c>
       <c r="BE3">
-        <v>54677438</v>
+        <v>12559164</v>
       </c>
       <c r="BF3">
-        <v>10541701</v>
+        <v>12917768</v>
       </c>
       <c r="BG3">
-        <v>9106435</v>
+        <v>15230915</v>
       </c>
       <c r="BH3">
-        <v>55173962</v>
+        <v>5749824</v>
       </c>
       <c r="BI3">
-        <v>12045156</v>
+        <v>12576863</v>
       </c>
       <c r="BJ3">
-        <v>12929595</v>
+        <v>11819609</v>
       </c>
       <c r="BK3">
-        <v>45864482</v>
+        <v>21684598</v>
       </c>
       <c r="BL3">
-        <v>8756328</v>
+        <v>16122981</v>
       </c>
       <c r="BM3">
-        <v>10992686</v>
+        <v>12405055</v>
       </c>
       <c r="BN3">
-        <v>8025234</v>
+        <v>9294538</v>
       </c>
       <c r="BO3">
-        <v>45418546</v>
+        <v>17436511</v>
       </c>
       <c r="BP3">
-        <v>8796815</v>
+        <v>9231499</v>
       </c>
       <c r="BQ3">
-        <v>17170707</v>
+        <v>7865486</v>
       </c>
       <c r="BR3">
-        <v>10258250</v>
+        <v>9736163</v>
       </c>
       <c r="BS3">
-        <v>18579886</v>
+        <v>8704057</v>
       </c>
       <c r="BT3">
-        <v>44360200</v>
+        <v>17426814</v>
       </c>
       <c r="BU3">
-        <v>36321415</v>
+        <v>13628446</v>
       </c>
       <c r="BV3">
-        <v>11993548</v>
+        <v>14364795</v>
       </c>
       <c r="BW3">
-        <v>49727807</v>
+        <v>11510565</v>
       </c>
       <c r="BX3">
-        <v>7522157</v>
-      </c>
-      <c r="BY3">
-        <v>7523813</v>
-      </c>
-      <c r="BZ3">
-        <v>14002461</v>
-      </c>
-      <c r="CA3">
-        <v>50151435</v>
-      </c>
-      <c r="CB3">
-        <v>24062407</v>
-      </c>
-      <c r="CC3">
-        <v>42946646</v>
-      </c>
-      <c r="CD3">
-        <v>40157330</v>
-      </c>
-      <c r="CE3">
-        <v>6514265</v>
-      </c>
-      <c r="CF3">
-        <v>9523452</v>
-      </c>
-      <c r="CG3">
-        <v>7892769</v>
-      </c>
-      <c r="CH3">
-        <v>8517468</v>
-      </c>
-      <c r="CI3">
-        <v>12559164</v>
-      </c>
-      <c r="CJ3">
-        <v>51760245</v>
-      </c>
-      <c r="CK3">
-        <v>12917768</v>
-      </c>
-      <c r="CL3">
-        <v>7867722</v>
-      </c>
-      <c r="CM3">
-        <v>24760306</v>
-      </c>
-      <c r="CN3">
-        <v>15230915</v>
-      </c>
-      <c r="CO3">
-        <v>5749824</v>
-      </c>
-      <c r="CP3">
-        <v>12576863</v>
-      </c>
-      <c r="CQ3">
-        <v>11819609</v>
-      </c>
-      <c r="CR3">
-        <v>21684598</v>
-      </c>
-      <c r="CS3">
-        <v>16122981</v>
-      </c>
-      <c r="CT3">
-        <v>12405055</v>
-      </c>
-      <c r="CU3">
-        <v>22794338</v>
-      </c>
-      <c r="CV3">
-        <v>9294538</v>
-      </c>
-      <c r="CW3">
-        <v>17436511</v>
-      </c>
-      <c r="CX3">
-        <v>9231499</v>
-      </c>
-      <c r="CY3">
-        <v>7865486</v>
-      </c>
-      <c r="CZ3">
-        <v>9736163</v>
-      </c>
-      <c r="DA3">
-        <v>8704057</v>
-      </c>
-      <c r="DB3">
-        <v>17426814</v>
-      </c>
-      <c r="DC3">
-        <v>13628446</v>
-      </c>
-      <c r="DD3">
-        <v>14364795</v>
-      </c>
-      <c r="DE3">
-        <v>11510565</v>
-      </c>
-      <c r="DF3">
         <v>11428352</v>
       </c>
     </row>

</xml_diff>